<commit_message>
updated e-manuscripta: get data from input file, not OAI interface
</commit_message>
<xml_diff>
--- a/e-manuscripta/e-manuscripta.xlsx
+++ b/e-manuscripta/e-manuscripta.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HeimK\switchdrive\dlza\e-manuscripta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HeimK\switchdrive\dlza\dlza\e-manuscripta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ADBFAA7-2571-46E8-9471-F865677F1E40}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB0A7D9C-539C-4F13-AF14-4D7FD41B2751}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="11750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="162">
   <si>
     <t/>
   </si>
@@ -31,27 +31,15 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Language</t>
-  </si>
-  <si>
-    <t>Record number</t>
-  </si>
-  <si>
     <t>MMS ID</t>
   </si>
   <si>
     <t>Catalogus plantarum circa Lucernam Helvetiorum sponte nascentium Carl Nicolaus Lang</t>
   </si>
   <si>
-    <t>Latin</t>
-  </si>
-  <si>
     <t>(HAN)000190119DSV05</t>
   </si>
   <si>
-    <t>German</t>
-  </si>
-  <si>
     <t>9914249335105505</t>
   </si>
   <si>
@@ -380,13 +368,154 @@
   </si>
   <si>
     <t>(1737.09.18.)</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-1</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-19</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-18</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-4</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-11</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-17</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-16</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-2</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-3</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-5</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-6</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-7</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-8</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-9</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-10</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-12</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-13</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-14</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Ms\emanus_Ms.40.4-3</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Ms\emanus_Ms.40.4-4</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Ms\emanus_Ms.60.fol</t>
+  </si>
+  <si>
+    <t>G:\ZHB-Sosa_Digital\digital\Ms\emanus_Ms.307.4</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24104</t>
+  </si>
+  <si>
+    <t>DOI</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24479</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24545</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-25099</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23616</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24491</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24544</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24546</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23892</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23621</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-25384</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24480</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23617</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23309</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-25216</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23742</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23620</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-25217</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23891</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-24105</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-23310</t>
+  </si>
+  <si>
+    <t>10.7891/e-manuscripta-108732</t>
+  </si>
+  <si>
+    <t>HAN number</t>
+  </si>
+  <si>
+    <t>Path</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -398,6 +527,11 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -425,7 +559,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -441,6 +575,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -863,546 +1006,623 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.54296875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="13.81640625" customWidth="1"/>
-    <col min="3" max="3" width="108.26953125" customWidth="1"/>
-    <col min="4" max="7" width="27.36328125" customWidth="1"/>
+    <col min="1" max="1" width="24.36328125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="18.08984375" customWidth="1"/>
+    <col min="3" max="3" width="77" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+    <col min="5" max="5" width="27.36328125" customWidth="1"/>
+    <col min="6" max="6" width="27.36328125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="48.54296875" customWidth="1"/>
+    <col min="8" max="8" width="28.1796875" customWidth="1"/>
+    <col min="9" max="9" width="46.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9">
       <c r="A1" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>134</v>
+      </c>
+      <c r="H2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="58">
+      <c r="A3" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>116</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="I3" s="9"/>
+    </row>
+    <row r="4" spans="1:9" ht="29">
+      <c r="A4" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>117</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="I4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" ht="58">
+      <c r="A5" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>118</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="43.5">
+      <c r="A6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" t="s">
+        <v>119</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="72.5">
+      <c r="A7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" t="s">
+        <v>121</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="29">
+      <c r="A9" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" t="s">
+        <v>122</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="29">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="G10" t="s">
+        <v>135</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="43.5">
+      <c r="A11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>130</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="58">
+      <c r="A12" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="58">
+      <c r="A13" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="43.5">
+      <c r="A14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" t="s">
+        <v>131</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="72.5">
+      <c r="A15" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="43.5">
+      <c r="A16" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G16" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="43.5">
+      <c r="A17" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="58">
+      <c r="A18" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" t="s">
+        <v>128</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="58">
+      <c r="A19" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="G19" t="s">
+        <v>125</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="101.5">
+      <c r="A20" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="116">
+      <c r="A21" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G21" t="s">
+        <v>133</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="43.5">
+      <c r="A22" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="29">
+      <c r="A23" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F19" s="1" t="s">
+      <c r="C23" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G19" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="87" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A22" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="C22" s="1" t="s">
+      <c r="F23" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>71</v>
+      <c r="G23" t="s">
+        <v>136</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H23" xr:uid="{8EDCE269-DDB7-4AA6-9846-DB04248D4CAF}"/>
+  <autoFilter ref="A1:H23" xr:uid="{3CBC698F-7B31-40D2-ADE1-34A45EAF21B5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
e-manuscripta: added identifier prefix, IIIF Metadata download
</commit_message>
<xml_diff>
--- a/e-manuscripta/e-manuscripta.xlsx
+++ b/e-manuscripta/e-manuscripta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HeimK\switchdrive\dlza\dlza\e-manuscripta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C23C5B9-BB29-49A4-8EF4-92017B71BD0C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F48E6C4-1670-4E1F-9E27-B0FE252D5E26}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6930" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,17 +16,14 @@
     <sheet name="results" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">results!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">results!$A$1:$F$23</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="154">
-  <si>
-    <t/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="155">
   <si>
     <t>Title</t>
   </si>
@@ -232,54 +229,6 @@
     <t>9914249310305505</t>
   </si>
   <si>
-    <t>Basel [1749-1751?]</t>
-  </si>
-  <si>
-    <t>Mitte 18. Jh.</t>
-  </si>
-  <si>
-    <t>1737.07.20.</t>
-  </si>
-  <si>
-    <t>1739?</t>
-  </si>
-  <si>
-    <t>1. Hälfte 18. Jh.</t>
-  </si>
-  <si>
-    <t>1736.04.19-05.25</t>
-  </si>
-  <si>
-    <t>1738.07.28.</t>
-  </si>
-  <si>
-    <t>1737.01.26.</t>
-  </si>
-  <si>
-    <t>1738.11.20.</t>
-  </si>
-  <si>
-    <t>1737.09.02.</t>
-  </si>
-  <si>
-    <t>1739.02.10.</t>
-  </si>
-  <si>
-    <t>1738.05.31.</t>
-  </si>
-  <si>
-    <t>1735.09.23.</t>
-  </si>
-  <si>
-    <t>1726?</t>
-  </si>
-  <si>
-    <t>1737.09.18.</t>
-  </si>
-  <si>
-    <t>Created</t>
-  </si>
-  <si>
     <t>Ms.307.4</t>
   </si>
   <si>
@@ -485,13 +434,67 @@
   </si>
   <si>
     <t>G:\ZHB-Sosa_Digital\digital\Pp\emanus_Pp.22.4-10</t>
+  </si>
+  <si>
+    <t>(HAN)none</t>
+  </si>
+  <si>
+    <t>e-manuscripta ID</t>
+  </si>
+  <si>
+    <t>1040365</t>
+  </si>
+  <si>
+    <t>1085689</t>
+  </si>
+  <si>
+    <t>1085764</t>
+  </si>
+  <si>
+    <t>1037517</t>
+  </si>
+  <si>
+    <t>1087850</t>
+  </si>
+  <si>
+    <t>1037375</t>
+  </si>
+  <si>
+    <t>1041431</t>
+  </si>
+  <si>
+    <t>1044448</t>
+  </si>
+  <si>
+    <t>1065627</t>
+  </si>
+  <si>
+    <t>1070683</t>
+  </si>
+  <si>
+    <t>1065720</t>
+  </si>
+  <si>
+    <t>1082162</t>
+  </si>
+  <si>
+    <t>1050314</t>
+  </si>
+  <si>
+    <t>1070517</t>
+  </si>
+  <si>
+    <t>1064072</t>
+  </si>
+  <si>
+    <t>1070442</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -504,13 +507,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color indexed="8"/>
-      <name val="Arial Unicode MS"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -520,12 +518,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="22"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -541,7 +533,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -553,13 +545,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -587,7 +576,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>273050</xdr:rowOff>
@@ -636,7 +625,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>946150</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>273050</xdr:rowOff>
@@ -982,553 +971,553 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.81640625" customWidth="1"/>
-    <col min="2" max="2" width="59.26953125" customWidth="1"/>
-    <col min="3" max="4" width="27.36328125" customWidth="1"/>
-    <col min="5" max="5" width="27.36328125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="27.36328125" customWidth="1"/>
+    <col min="1" max="1" width="59.28515625" customWidth="1"/>
+    <col min="2" max="3" width="27.42578125" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" customWidth="1"/>
+    <col min="6" max="6" width="27.42578125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="29">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="E1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="29">
-      <c r="A2" s="3" t="s">
-        <v>69</v>
-      </c>
       <c r="B2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="3">
+        <v>3120805</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="29">
-      <c r="A3" s="3">
-        <v>1723</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1060335</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="72.5">
-      <c r="A4" s="3">
-        <v>1740</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="G4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="29">
-      <c r="A5" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="G5" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="72.5">
-      <c r="A6" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="58">
-      <c r="A7" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1040251</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-    </row>
-    <row r="8" spans="1:10" ht="87">
-      <c r="A8" s="3">
-        <v>1737</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="G8" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G9" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="43.5">
-      <c r="A10" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G10" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="43.5">
-      <c r="A11" s="3">
-        <v>1748</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1050665</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="G11" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="58">
-      <c r="A12" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F12" s="3">
+        <v>1041555</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="G12" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="72.5">
-      <c r="A13" s="3" t="s">
-        <v>75</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G13" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="72.5">
-      <c r="A14" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="58">
-      <c r="A15" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="G15" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="87">
-      <c r="A16" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="G16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="58">
-      <c r="A17" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="G17" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="58">
-      <c r="A18" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="G18" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="72.5">
-      <c r="A19" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="G19" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="72.5">
-      <c r="A20" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="150" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G20" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="130.5">
-      <c r="A21" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="180" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="G21" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="159.5">
-      <c r="A22" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F22" s="3">
+        <v>1060398</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="G22" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="58">
-      <c r="A23" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="G23" t="s">
-        <v>153</v>
+      <c r="E23" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G23" xr:uid="{70F860E9-B47E-4046-8DA0-219C65757750}"/>
+  <autoFilter ref="A1:F23" xr:uid="{70F860E9-B47E-4046-8DA0-219C65757750}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="E2:E23" numberStoredAsText="1"/>
+    <ignoredError sqref="D3:D23" numberStoredAsText="1"/>
   </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>